<commit_message>
Updated controls in database and proper integration with database NIshant
</commit_message>
<xml_diff>
--- a/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
+++ b/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFADE2B3-705E-4D2F-A8F8-E658C402A4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD0FE8FA-B0F1-4AAB-840B-833F113BF457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-106" yWindow="-106" windowWidth="18644" windowHeight="9879" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="130">
   <si>
     <t>S.No</t>
   </si>
@@ -436,12 +436,30 @@
   <si>
     <t>SEBI/CERT-In reporting evidence; templates</t>
   </si>
+  <si>
+    <t>Audit_Framwork</t>
+  </si>
+  <si>
+    <t>Audit_Category</t>
+  </si>
+  <si>
+    <t>Audit_subcategory</t>
+  </si>
+  <si>
+    <t>AIF</t>
+  </si>
+  <si>
+    <t>self-certified</t>
+  </si>
+  <si>
+    <t>SEBI-CSCRF</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,8 +479,27 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -475,8 +512,14 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -499,17 +542,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -784,14 +853,16 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="7" max="7" width="19.25" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="25.95" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="25.95" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -803,12 +874,20 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -825,9 +904,17 @@
         <v>9</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="184.35" x14ac:dyDescent="0.35">
+      <c r="G2" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="184.35" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -846,9 +933,17 @@
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G3" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -865,9 +960,17 @@
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -886,9 +989,17 @@
       <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G5" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -905,9 +1016,17 @@
         <v>23</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -924,9 +1043,17 @@
         <v>27</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -945,9 +1072,17 @@
       <c r="F8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="230.4" x14ac:dyDescent="0.35">
+      <c r="G8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="230.4" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -966,9 +1101,17 @@
       <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -987,9 +1130,17 @@
       <c r="F10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="161.30000000000001" x14ac:dyDescent="0.35">
+      <c r="G10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="161.30000000000001" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1008,9 +1159,17 @@
       <c r="F11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1029,9 +1188,17 @@
       <c r="F12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G12" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1050,9 +1217,17 @@
       <c r="F13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G13" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1071,9 +1246,17 @@
       <c r="F14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" ht="322.60000000000002" x14ac:dyDescent="0.35">
+      <c r="G14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="334.1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1092,9 +1275,17 @@
       <c r="F15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1113,9 +1304,17 @@
       <c r="F16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1134,9 +1333,17 @@
       <c r="F17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G17" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1155,9 +1362,17 @@
       <c r="F18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G18" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1176,9 +1391,17 @@
       <c r="F19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1197,9 +1420,17 @@
       <c r="F20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G20" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1218,9 +1449,17 @@
       <c r="F21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" ht="103.7" x14ac:dyDescent="0.35">
+      <c r="G21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="103.7" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1239,9 +1478,17 @@
       <c r="F22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G22" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1260,9 +1507,17 @@
       <c r="F23" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G23" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1281,9 +1536,17 @@
       <c r="F24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G24" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1302,9 +1565,17 @@
       <c r="F25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G25" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1323,9 +1594,17 @@
       <c r="F26" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1344,9 +1623,17 @@
       <c r="F27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G27" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1365,9 +1652,17 @@
       <c r="F28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G28" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1386,9 +1681,17 @@
       <c r="F29" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G29" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1407,7 +1710,15 @@
       <c r="F30" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="G30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>128</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
backend updated v4 Nishant
</commit_message>
<xml_diff>
--- a/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
+++ b/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFADE2B3-705E-4D2F-A8F8-E658C402A4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD0FE8FA-B0F1-4AAB-840B-833F113BF457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-106" yWindow="-106" windowWidth="18644" windowHeight="9879" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="130">
   <si>
     <t>S.No</t>
   </si>
@@ -436,12 +436,30 @@
   <si>
     <t>SEBI/CERT-In reporting evidence; templates</t>
   </si>
+  <si>
+    <t>Audit_Framwork</t>
+  </si>
+  <si>
+    <t>Audit_Category</t>
+  </si>
+  <si>
+    <t>Audit_subcategory</t>
+  </si>
+  <si>
+    <t>AIF</t>
+  </si>
+  <si>
+    <t>self-certified</t>
+  </si>
+  <si>
+    <t>SEBI-CSCRF</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,8 +479,27 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -475,8 +512,14 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -499,17 +542,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -784,14 +853,16 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="7" max="7" width="19.25" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="25.95" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="25.95" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -803,12 +874,20 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -825,9 +904,17 @@
         <v>9</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="184.35" x14ac:dyDescent="0.35">
+      <c r="G2" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="184.35" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -846,9 +933,17 @@
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G3" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -865,9 +960,17 @@
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -886,9 +989,17 @@
       <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G5" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -905,9 +1016,17 @@
         <v>23</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -924,9 +1043,17 @@
         <v>27</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -945,9 +1072,17 @@
       <c r="F8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="230.4" x14ac:dyDescent="0.35">
+      <c r="G8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="230.4" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -966,9 +1101,17 @@
       <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -987,9 +1130,17 @@
       <c r="F10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="161.30000000000001" x14ac:dyDescent="0.35">
+      <c r="G10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="161.30000000000001" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1008,9 +1159,17 @@
       <c r="F11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1029,9 +1188,17 @@
       <c r="F12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G12" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1050,9 +1217,17 @@
       <c r="F13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G13" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1071,9 +1246,17 @@
       <c r="F14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" ht="322.60000000000002" x14ac:dyDescent="0.35">
+      <c r="G14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="334.1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1092,9 +1275,17 @@
       <c r="F15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1113,9 +1304,17 @@
       <c r="F16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1134,9 +1333,17 @@
       <c r="F17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G17" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1155,9 +1362,17 @@
       <c r="F18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G18" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1176,9 +1391,17 @@
       <c r="F19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1197,9 +1420,17 @@
       <c r="F20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G20" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1218,9 +1449,17 @@
       <c r="F21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" ht="103.7" x14ac:dyDescent="0.35">
+      <c r="G21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="103.7" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1239,9 +1478,17 @@
       <c r="F22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G22" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1260,9 +1507,17 @@
       <c r="F23" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G23" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1281,9 +1536,17 @@
       <c r="F24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G24" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1302,9 +1565,17 @@
       <c r="F25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G25" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1323,9 +1594,17 @@
       <c r="F26" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1344,9 +1623,17 @@
       <c r="F27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G27" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1365,9 +1652,17 @@
       <c r="F28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G28" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1386,9 +1681,17 @@
       <c r="F29" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G29" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1407,7 +1710,15 @@
       <c r="F30" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="G30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>128</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
backend files updated for controls Nishant v4
</commit_message>
<xml_diff>
--- a/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
+++ b/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFADE2B3-705E-4D2F-A8F8-E658C402A4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD0FE8FA-B0F1-4AAB-840B-833F113BF457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-106" yWindow="-106" windowWidth="18644" windowHeight="9879" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="130">
   <si>
     <t>S.No</t>
   </si>
@@ -436,12 +436,30 @@
   <si>
     <t>SEBI/CERT-In reporting evidence; templates</t>
   </si>
+  <si>
+    <t>Audit_Framwork</t>
+  </si>
+  <si>
+    <t>Audit_Category</t>
+  </si>
+  <si>
+    <t>Audit_subcategory</t>
+  </si>
+  <si>
+    <t>AIF</t>
+  </si>
+  <si>
+    <t>self-certified</t>
+  </si>
+  <si>
+    <t>SEBI-CSCRF</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,8 +479,27 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -475,8 +512,14 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -499,17 +542,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -784,14 +853,16 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="7" max="7" width="19.25" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="25.95" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="25.95" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -803,12 +874,20 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -825,9 +904,17 @@
         <v>9</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="184.35" x14ac:dyDescent="0.35">
+      <c r="G2" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="184.35" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -846,9 +933,17 @@
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G3" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -865,9 +960,17 @@
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -886,9 +989,17 @@
       <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G5" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -905,9 +1016,17 @@
         <v>23</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -924,9 +1043,17 @@
         <v>27</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -945,9 +1072,17 @@
       <c r="F8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="230.4" x14ac:dyDescent="0.35">
+      <c r="G8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="230.4" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -966,9 +1101,17 @@
       <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -987,9 +1130,17 @@
       <c r="F10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="161.30000000000001" x14ac:dyDescent="0.35">
+      <c r="G10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="161.30000000000001" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1008,9 +1159,17 @@
       <c r="F11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1029,9 +1188,17 @@
       <c r="F12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G12" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1050,9 +1217,17 @@
       <c r="F13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G13" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1071,9 +1246,17 @@
       <c r="F14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" ht="322.60000000000002" x14ac:dyDescent="0.35">
+      <c r="G14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="334.1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1092,9 +1275,17 @@
       <c r="F15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1113,9 +1304,17 @@
       <c r="F16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1134,9 +1333,17 @@
       <c r="F17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G17" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1155,9 +1362,17 @@
       <c r="F18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G18" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1176,9 +1391,17 @@
       <c r="F19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1197,9 +1420,17 @@
       <c r="F20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G20" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1218,9 +1449,17 @@
       <c r="F21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" ht="103.7" x14ac:dyDescent="0.35">
+      <c r="G21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="103.7" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1239,9 +1478,17 @@
       <c r="F22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G22" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1260,9 +1507,17 @@
       <c r="F23" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G23" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1281,9 +1536,17 @@
       <c r="F24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G24" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1302,9 +1565,17 @@
       <c r="F25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G25" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1323,9 +1594,17 @@
       <c r="F26" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1344,9 +1623,17 @@
       <c r="F27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G27" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1365,9 +1652,17 @@
       <c r="F28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G28" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1386,9 +1681,17 @@
       <c r="F29" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G29" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1407,7 +1710,15 @@
       <c r="F30" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="G30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>128</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
flaws corrected pulled from main-demo
</commit_message>
<xml_diff>
--- a/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
+++ b/backend/app/data/controls/AIF_Controls_Self_Certified_RE.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFADE2B3-705E-4D2F-A8F8-E658C402A4F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD0FE8FA-B0F1-4AAB-840B-833F113BF457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-106" yWindow="-106" windowWidth="18644" windowHeight="9879" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="130">
   <si>
     <t>S.No</t>
   </si>
@@ -436,12 +436,30 @@
   <si>
     <t>SEBI/CERT-In reporting evidence; templates</t>
   </si>
+  <si>
+    <t>Audit_Framwork</t>
+  </si>
+  <si>
+    <t>Audit_Category</t>
+  </si>
+  <si>
+    <t>Audit_subcategory</t>
+  </si>
+  <si>
+    <t>AIF</t>
+  </si>
+  <si>
+    <t>self-certified</t>
+  </si>
+  <si>
+    <t>SEBI-CSCRF</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -461,8 +479,27 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -475,8 +512,14 @@
         <bgColor rgb="FF003366"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -499,17 +542,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -775,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -784,14 +853,16 @@
     <col min="4" max="4" width="60" customWidth="1"/>
     <col min="5" max="5" width="35" customWidth="1"/>
     <col min="6" max="6" width="40" customWidth="1"/>
-    <col min="8" max="8" width="40" customWidth="1"/>
+    <col min="7" max="7" width="19.25" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
+    <col min="9" max="9" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="25.95" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="25.95" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -803,12 +874,20 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="1"/>
-    </row>
-    <row r="2" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G1" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -825,9 +904,17 @@
         <v>9</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="H2" s="2"/>
-    </row>
-    <row r="3" spans="1:8" ht="184.35" x14ac:dyDescent="0.35">
+      <c r="G2" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="184.35" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -846,9 +933,17 @@
       <c r="F3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G3" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I3" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -865,9 +960,17 @@
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G4" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H4" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -886,9 +989,17 @@
       <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="2"/>
-    </row>
-    <row r="6" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G5" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -905,9 +1016,17 @@
         <v>23</v>
       </c>
       <c r="F6" s="2"/>
-      <c r="H6" s="2"/>
-    </row>
-    <row r="7" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -924,9 +1043,17 @@
         <v>27</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G7" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -945,9 +1072,17 @@
       <c r="F8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="230.4" x14ac:dyDescent="0.35">
+      <c r="G8" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="230.4" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -966,9 +1101,17 @@
       <c r="F9" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G9" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -987,9 +1130,17 @@
       <c r="F10" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:8" ht="161.30000000000001" x14ac:dyDescent="0.35">
+      <c r="G10" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="161.30000000000001" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1008,9 +1159,17 @@
       <c r="F11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G11" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1029,9 +1188,17 @@
       <c r="F12" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G12" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1050,9 +1217,17 @@
       <c r="F13" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G13" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1071,9 +1246,17 @@
       <c r="F14" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="H14" s="2"/>
-    </row>
-    <row r="15" spans="1:8" ht="322.60000000000002" x14ac:dyDescent="0.35">
+      <c r="G14" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="334.1" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1092,9 +1275,17 @@
       <c r="F15" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G15" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1113,9 +1304,17 @@
       <c r="F16" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G16" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1134,9 +1333,17 @@
       <c r="F17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="H17" s="2"/>
-    </row>
-    <row r="18" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G17" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1155,9 +1362,17 @@
       <c r="F18" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="H18" s="2"/>
-    </row>
-    <row r="19" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G18" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1176,9 +1391,17 @@
       <c r="F19" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="H19" s="2"/>
-    </row>
-    <row r="20" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G19" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1197,9 +1420,17 @@
       <c r="F20" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="H20" s="2"/>
-    </row>
-    <row r="21" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G20" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1218,9 +1449,17 @@
       <c r="F21" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H21" s="2"/>
-    </row>
-    <row r="22" spans="1:8" ht="103.7" x14ac:dyDescent="0.35">
+      <c r="G21" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="103.7" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1239,9 +1478,17 @@
       <c r="F22" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="H22" s="2"/>
-    </row>
-    <row r="23" spans="1:8" ht="46.1" x14ac:dyDescent="0.35">
+      <c r="G22" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="46.1" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1260,9 +1507,17 @@
       <c r="F23" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="H23" s="2"/>
-    </row>
-    <row r="24" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G23" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1281,9 +1536,17 @@
       <c r="F24" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="H24" s="2"/>
-    </row>
-    <row r="25" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G24" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1302,9 +1565,17 @@
       <c r="F25" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H25" s="2"/>
-    </row>
-    <row r="26" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G25" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -1323,9 +1594,17 @@
       <c r="F26" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H26" s="2"/>
-    </row>
-    <row r="27" spans="1:8" ht="69.150000000000006" x14ac:dyDescent="0.35">
+      <c r="G26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="69.150000000000006" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -1344,9 +1623,17 @@
       <c r="F27" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="H27" s="2"/>
-    </row>
-    <row r="28" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G27" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -1365,9 +1652,17 @@
       <c r="F28" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="H28" s="2"/>
-    </row>
-    <row r="29" spans="1:8" ht="34.6" x14ac:dyDescent="0.35">
+      <c r="G28" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="34.6" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1386,9 +1681,17 @@
       <c r="F29" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="H29" s="2"/>
-    </row>
-    <row r="30" spans="1:8" ht="23.05" x14ac:dyDescent="0.35">
+      <c r="G29" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="23.05" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -1407,7 +1710,15 @@
       <c r="F30" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="H30" s="2"/>
+      <c r="G30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H30" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>128</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>

</xml_diff>